<commit_message>
Price update and final BOM
The actual prices were added as an image of the order placed, and the BOM downloaded directly from the order was added.
</commit_message>
<xml_diff>
--- a/pcb/robot/usb-pd-module/USB_PD_Module_BOM.xlsx
+++ b/pcb/robot/usb-pd-module/USB_PD_Module_BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JHORDAN\FREELANCE\PROYECTOS\KICAD_USB_PD_MODULAR\Github\smartphone-robot-cad\pcb\robot\usb-pd-module\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA19E2AD-F65F-4F97-B000-E668666198BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD8FC6BD-3A8F-47F7-867B-8DFDD6C4D706}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="84">
   <si>
     <t>Footprint</t>
   </si>
@@ -306,6 +306,12 @@
   </si>
   <si>
     <t>RC0603JR-07120KL</t>
+  </si>
+  <si>
+    <t>RC0402FR-07100RL</t>
+  </si>
+  <si>
+    <t>RC0402FR-07422RL</t>
   </si>
 </sst>
 </file>
@@ -850,7 +856,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -861,7 +867,9 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -926,22 +934,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>285750</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>81644</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>553910</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>10111</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>610921</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>159724</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8341EDA9-660D-4292-BA42-7D0C2C5726FD}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{36443C27-EBEC-4777-AC76-3C9D1328A0AE}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -957,8 +965,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7772400" y="1362075"/>
-          <a:ext cx="10459910" cy="4201111"/>
+          <a:off x="8749393" y="1251858"/>
+          <a:ext cx="9469171" cy="3724795"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1272,8 +1280,10 @@
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" customWidth="1"/>
+    <col min="3" max="3" width="29.28515625" customWidth="1"/>
     <col min="4" max="4" width="27.85546875" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.75">
@@ -1289,6 +1299,8 @@
       <c r="D1" s="2" t="s">
         <v>71</v>
       </c>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
@@ -1303,8 +1315,8 @@
       <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
@@ -1319,8 +1331,8 @@
       <c r="D3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3" t="s">
@@ -1335,8 +1347,8 @@
       <c r="D4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3" t="s">
@@ -1351,8 +1363,8 @@
       <c r="D5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
     </row>
     <row r="6" spans="1:6" ht="16.5">
       <c r="A6" s="5" t="s">
@@ -1367,10 +1379,10 @@
       <c r="D6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="8">
         <v>2188470001</v>
       </c>
     </row>
@@ -1387,10 +1399,10 @@
       <c r="D7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:6" ht="16.5">
       <c r="A8" s="3">
         <v>100</v>
       </c>
@@ -1400,11 +1412,13 @@
       <c r="C8" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="3"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="D8" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:6" ht="16.5">
       <c r="A9" s="3">
         <v>422</v>
       </c>
@@ -1414,9 +1428,11 @@
       <c r="C9" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="3"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
+      <c r="D9" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="3" t="s">
@@ -1431,8 +1447,8 @@
       <c r="D10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="5">
@@ -1447,10 +1463,10 @@
       <c r="D11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="5" t="s">
         <v>78</v>
       </c>
     </row>
@@ -1467,8 +1483,8 @@
       <c r="D12" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="5" t="s">
@@ -1483,10 +1499,10 @@
       <c r="D13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="5" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1503,10 +1519,10 @@
       <c r="D14" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="5" t="s">
         <v>80</v>
       </c>
     </row>
@@ -1523,10 +1539,10 @@
       <c r="D15" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="5" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1543,8 +1559,8 @@
       <c r="D16" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="3">
@@ -1559,8 +1575,8 @@
       <c r="D17" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="3">
@@ -1575,8 +1591,8 @@
       <c r="D18" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="3" t="s">
@@ -1591,8 +1607,8 @@
       <c r="D19" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="3" t="s">
@@ -1604,11 +1620,11 @@
       <c r="C20" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="3" t="s">
@@ -1623,8 +1639,8 @@
       <c r="D21" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="3" t="s">
@@ -1639,8 +1655,8 @@
       <c r="D22" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="3" t="s">
@@ -1655,8 +1671,8 @@
       <c r="D23" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="3" t="s">
@@ -1671,8 +1687,8 @@
       <c r="D24" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="3" t="s">
@@ -1687,8 +1703,8 @@
       <c r="D25" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="4"/>

</xml_diff>